<commit_message>
feat: verify geometry identity too when detecting folder-duplicate layers
</commit_message>
<xml_diff>
--- a/work1-ledger-cleanup/fill_rate_report.xlsx
+++ b/work1-ledger-cleanup/fill_rate_report.xlsx
@@ -538,7 +538,7 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>汚水フォルダと同一データ(差はエクスポート日時列のみ)</t>
+          <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restore layer names from the distribution's layer.xml in the inventory
</commit_message>
<xml_diff>
--- a/work1-ledger-cleanup/fill_rate_report.xlsx
+++ b/work1-ledger-cleanup/fill_rate_report.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>マンホール注記</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>マンホール引出線</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -778,7 +778,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠注記</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠引出線</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -934,7 +934,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>桝注記</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠断面シンボル</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠勾配シンボル</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>副管</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠記号（副管）</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠記号（起点）</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>副管</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠記号（副管）</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管渠記号（起点）</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水マンホール注記</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水マンホール引出線</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水管渠引出線</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水管渠注記</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水管渠断面シンボル</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水管渠勾配シンボル</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>雨水桝注記</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管路区切</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>(配布物に名称なし)</t>
+          <t>管路注記</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: make report sheets print-ready and size columns by display width
Shared style_sheet() in the four report-writing tools now:
- sizes columns counting CJK glyphs as two units (len() under-sized
  Japanese headers)
- sets A4 landscape, fit-to-width, and repeats the header row on every
  printed page
fill_rate_report reuses the same function instead of an inline loop.
</commit_message>
<xml_diff>
--- a/work1-ledger-cleanup/fill_rate_report.xlsx
+++ b/work1-ledger-cleanup/fill_rate_report.xlsx
@@ -11,7 +11,11 @@
     <sheet name="レイヤ棚卸し" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="属性記入率" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'サマリ'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'レイヤ棚卸し'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'属性記入率'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -425,13 +429,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,6 +522,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -525,20 +530,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="39" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1944,6 +1949,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1951,18 +1957,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5861,5 +5867,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: print gridlines, run dates, and source URLs in report workbooks
- style_sheet: print gridlines (screen gridlines are not printed by
  default, which leaves rows floating on paper)
- ledger_qa / fill_rate_report: record the run date in the summary sheet
- judge_urgency: the criteria sheet now resolves each source label to the
  document title and URL from criteria["sources"]
</commit_message>
<xml_diff>
--- a/work1-ledger-cleanup/fill_rate_report.xlsx
+++ b/work1-ledger-cleanup/fill_rate_report.xlsx
@@ -431,11 +431,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,74 +453,87 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>配布ファイル数</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>34</v>
+          <t>集計実行日</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>実質レイヤ数(重複を除く)</t>
+          <t>配布ファイル数</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>うち業務属性を持つレイヤ</t>
+          <t>実質レイヤ数(重複を除く)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>検査した属性数</t>
+          <t>うち業務属性を持つレイヤ</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>133</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>記入率90%以上の属性</t>
+          <t>検査した属性数</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>48</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>記入率10%未満の属性</t>
+          <t>記入率90%以上の属性</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>記入率10%未満の属性</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>記入率0%(全件空)の属性</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>49</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1948,6 +1961,7 @@
       <c r="I35" t="inlineStr"/>
     </row>
   </sheetData>
+  <printOptions gridLines="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5866,6 +5880,7 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: wrap long text columns, write run dates as dates, link source URLs
- style_sheet: columns that hit max_width get wrap_text so long text
  (e.g. 判定根拠) prints in full instead of being clipped
- summaries: run date is a real date cell (filterable), not an ISO string
- judge_urgency: 出典URL cells on the criteria sheet are hyperlinks
</commit_message>
<xml_diff>
--- a/work1-ledger-cleanup/fill_rate_report.xlsx
+++ b/work1-ledger-cleanup/fill_rate_report.xlsx
@@ -22,7 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -61,10 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,10 +463,8 @@
           <t>集計実行日</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="B2" s="2" t="n">
+        <v>46257</v>
       </c>
     </row>
     <row r="3">
@@ -643,7 +648,7 @@
           <t>マンホール</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -682,7 +687,7 @@
           <t>マンホール注記</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -721,7 +726,7 @@
           <t>マンホール引出線</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -760,7 +765,7 @@
           <t>管渠</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -799,7 +804,7 @@
           <t>管渠注記</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -838,7 +843,7 @@
           <t>管渠引出線</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -877,7 +882,7 @@
           <t>桝</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -916,7 +921,7 @@
           <t>取付管</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -955,7 +960,7 @@
           <t>桝注記</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -994,7 +999,7 @@
           <t>管渠断面シンボル</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1033,7 +1038,7 @@
           <t>管渠勾配シンボル</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1072,7 +1077,7 @@
           <t>副管</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1111,7 +1116,7 @@
           <t>管渠記号（副管）</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1150,7 +1155,7 @@
           <t>管渠記号（起点）</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1189,7 +1194,7 @@
           <t>マンホール</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1232,7 +1237,7 @@
           <t>管渠</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1275,7 +1280,7 @@
           <t>桝</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1318,7 +1323,7 @@
           <t>取付管</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1361,7 +1366,7 @@
           <t>副管</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1404,7 +1409,7 @@
           <t>管渠記号（副管）</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1447,7 +1452,7 @@
           <t>管渠記号（起点）</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>汚水フォルダと同一データ(図形一致・属性の差はエクスポート日時列のみ)</t>
         </is>
@@ -1490,7 +1495,7 @@
           <t>雨水マンホール注記</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1529,7 +1534,7 @@
           <t>雨水マンホール引出線</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1568,7 +1573,7 @@
           <t>雨水管渠引出線</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1607,7 +1612,7 @@
           <t>雨水管渠注記</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1646,7 +1651,7 @@
           <t>雨水管渠断面シンボル</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1685,7 +1690,7 @@
           <t>雨水管渠勾配シンボル</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1724,7 +1729,7 @@
           <t>雨水桝注記</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1763,7 +1768,7 @@
           <t>管路</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1802,7 +1807,7 @@
           <t>管路区切</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1841,7 +1846,7 @@
           <t>管路注記</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1880,7 +1885,7 @@
           <t>給水管</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1919,7 +1924,7 @@
           <t>弁栓</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1958,7 +1963,7 @@
           <t>消火栓</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions gridLines="1"/>

</xml_diff>